<commit_message>
copyright年号変更 (2025 -> 2026)
</commit_message>
<xml_diff>
--- a/xyz.hotchpotch.hogandiff/src/main/resources/result_book.xlsx
+++ b/xyz.hotchpotch.hogandiff/src/main/resources/result_book.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48fdcf04b383bd82/workspace_202412/hogandiff4/xyz.hotchpotch.hogandiff/src/main/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48fdcf04b383bd82/workspace_202509/hogandiff4/xyz.hotchpotch.hogandiff/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{4E3D4435-F909-422E-8C85-6F8A2F8AC702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FA932A7-6641-48A7-8A82-5B2367DA4ACC}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{4E3D4435-F909-422E-8C85-6F8A2F8AC702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{714BA601-54F8-4BEA-9826-28C57FA1B8E6}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22180" windowHeight="14140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="result" sheetId="3" r:id="rId1"/>
@@ -97,7 +97,7 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>方眼Diff © 2018-2025 nmby</t>
+    <t>方眼Diff © 2018-2026 nmby</t>
     <rPh sb="0" eb="2">
       <t>ホウガン</t>
     </rPh>
@@ -492,110 +492,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person0.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person1.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person10.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person11.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person12.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person13.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person14.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person15.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person16.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person17.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person18.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person19.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person2.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person20.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person21.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person22.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person23.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person24.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person3.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person4.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person5.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person6.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person7.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person8.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/persons/person9.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -866,15 +762,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="D1:H18"/>
-  <sheetFormatPr defaultColWidth="2.5625" defaultRowHeight="17.649999999999999"/>
+  <sheetFormatPr defaultColWidth="2.58203125" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="2" width="2.5625" style="1"/>
+    <col min="1" max="2" width="2.58203125" style="1"/>
     <col min="3" max="3" width="4" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.0625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="52.5625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.0625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="52.5625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="2.5625" style="1"/>
+    <col min="4" max="4" width="8.08203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="52.58203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.08203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="52.58203125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="2.58203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="4:8">

</xml_diff>